<commit_message>
Map Sheet 1 material fields for ceiling, downpipes, and gutters.
Add sheet1_collective helper; fix appendix ceiling type; add material columns to Table 4-2; regenerate Brookton outputs.
</commit_message>
<xml_diff>
--- a/projects/26126 - Brookton DHS Demountable/output/tables/Table 4-2 Overall Condition of External Rooms and Components.xlsx
+++ b/projects/26126 - Brookton DHS Demountable/output/tables/Table 4-2 Overall Condition of External Rooms and Components.xlsx
@@ -92,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -104,6 +104,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -471,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -482,6 +485,9 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,30 +510,45 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
+          <t>External Walls Material</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
           <t>Downpipes</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Downpipes Material</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Gutters</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Gutters Material</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Roof</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Ramp</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>Subfloor Framing</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Windows</t>
         </is>
@@ -544,32 +565,47 @@
           <t>Fair</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Gyprock/ACM</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>Fair</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>PVC</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t>Fair</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Colorbond</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
         <is>
           <t>Fair</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Fair</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>Fair</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Fair</t>
         </is>
@@ -577,7 +613,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>